<commit_message>
Fix public repository URL spelling
</commit_message>
<xml_diff>
--- a/supplementary_tables/Supplementary_Tables_S1_S18.xlsx
+++ b/supplementary_tables/Supplementary_Tables_S1_S18.xlsx
@@ -9174,7 +9174,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>https://github.com/dchen0212/trimole_hybird/results_strict/case_study_v36_exact_full/full_predictions/ppbr_az/test_predictions_full_seed_mean.csv</t>
+          <t>https://github.com/dchen0212/trimole_hybrid/results_strict/case_study_v36_exact_full/full_predictions/ppbr_az/test_predictions_full_seed_mean.csv</t>
         </is>
       </c>
       <c r="Q2" t="n">
@@ -9419,7 +9419,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>https://github.com/dchen0212/trimole_hybird/results_strict/case_study_v36_exact_full/full_predictions/ppbr_az/test_predictions_full_seed_mean.csv</t>
+          <t>https://github.com/dchen0212/trimole_hybrid/results_strict/case_study_v36_exact_full/full_predictions/ppbr_az/test_predictions_full_seed_mean.csv</t>
         </is>
       </c>
       <c r="Q3" t="n">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>https://github.com/dchen0212/trimole_hybird/results_strict/case_study_v36_exact_full/full_predictions/clearance_hepatocyte_az/test_predictions_full_seed_mean.csv</t>
+          <t>https://github.com/dchen0212/trimole_hybrid/results_strict/case_study_v36_exact_full/full_predictions/clearance_hepatocyte_az/test_predictions_full_seed_mean.csv</t>
         </is>
       </c>
       <c r="Q4" t="n">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>https://github.com/dchen0212/trimole_hybird/results_strict/case_study_v36_exact_full/full_predictions/clearance_microsome_az/test_predictions_full_seed_mean.csv</t>
+          <t>https://github.com/dchen0212/trimole_hybrid/results_strict/case_study_v36_exact_full/full_predictions/clearance_microsome_az/test_predictions_full_seed_mean.csv</t>
         </is>
       </c>
       <c r="Q5" t="n">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>https://github.com/dchen0212/trimole_hybird/results_strict/case_study_v36_exact_full/full_predictions/vdss_lombardo/test_predictions_full_seed_mean.csv</t>
+          <t>https://github.com/dchen0212/trimole_hybrid/results_strict/case_study_v36_exact_full/full_predictions/vdss_lombardo/test_predictions_full_seed_mean.csv</t>
         </is>
       </c>
       <c r="Q6" t="n">
@@ -10417,7 +10417,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>https://github.com/dchen0212/trimole_hybird/results_strict/case_study_v36_exact_full/full_predictions/pgp_broccatelli/test_predictions_full_seed_mean.csv</t>
+          <t>https://github.com/dchen0212/trimole_hybrid/results_strict/case_study_v36_exact_full/full_predictions/pgp_broccatelli/test_predictions_full_seed_mean.csv</t>
         </is>
       </c>
       <c r="Q7" t="n">
@@ -10676,7 +10676,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>https://github.com/dchen0212/trimole_hybird/results_strict/case_study_v36_exact_full/full_predictions/hia_hou/test_predictions_full_seed_mean.csv</t>
+          <t>https://github.com/dchen0212/trimole_hybrid/results_strict/case_study_v36_exact_full/full_predictions/hia_hou/test_predictions_full_seed_mean.csv</t>
         </is>
       </c>
       <c r="Q8" t="n">
@@ -10935,7 +10935,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>https://github.com/dchen0212/trimole_hybird/results_strict/case_study_v36_exact_full/full_predictions/cyp3a4_substrate_carbonmangels/test_predictions_full_seed_mean.csv</t>
+          <t>https://github.com/dchen0212/trimole_hybrid/results_strict/case_study_v36_exact_full/full_predictions/cyp3a4_substrate_carbonmangels/test_predictions_full_seed_mean.csv</t>
         </is>
       </c>
       <c r="Q9" t="n">
@@ -11191,7 +11191,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>https://github.com/dchen0212/trimole_hybird/results_strict/case_study_v36_exact_full/full_predictions/caco2_wang/test_predictions_full_seed_mean.csv</t>
+          <t>https://github.com/dchen0212/trimole_hybrid/results_strict/case_study_v36_exact_full/full_predictions/caco2_wang/test_predictions_full_seed_mean.csv</t>
         </is>
       </c>
       <c r="Q10" t="n">
@@ -11436,7 +11436,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>https://github.com/dchen0212/trimole_hybird/results_strict/case_study_v36_exact_full/full_predictions/clearance_microsome_az/test_predictions_full_seed_mean.csv</t>
+          <t>https://github.com/dchen0212/trimole_hybrid/results_strict/case_study_v36_exact_full/full_predictions/clearance_microsome_az/test_predictions_full_seed_mean.csv</t>
         </is>
       </c>
       <c r="Q11" t="n">
@@ -41915,7 +41915,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://github.com/dchen0212/trimole_hybird</t>
+          <t>https://github.com/dchen0212/trimole_hybrid</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -41977,7 +41977,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://github.com/dchen0212/trimole_hybird</t>
+          <t>https://github.com/dchen0212/trimole_hybrid</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">

</xml_diff>